<commit_message>
feat: Mettre à jour le fichier Cahier de test.xlsx
</commit_message>
<xml_diff>
--- a/Cahier de test.xlsx
+++ b/Cahier de test.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miyu\Documents\Ecole\CDA\Conception solutions logicielles\Individuel\RENDU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miyu\Documents\Ecole\CDA\Conception solutions logicielles\Individuel\CESIZen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D7EA28-2AE3-4698-9F0C-60F74FCDF057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B0B8C2C-E4CF-417A-8DE7-48F3035DDEC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="3015" windowWidth="29040" windowHeight="15870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -594,10 +594,6 @@
         <f>"Responsable"</f>
         <v>Responsable</v>
       </c>
-      <c r="L1" s="8" t="str">
-        <f>"Date"</f>
-        <v>Date</v>
-      </c>
     </row>
     <row r="2" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="str">
@@ -755,7 +751,7 @@
         <v>AUTH-01</v>
       </c>
       <c r="B5" s="3" t="str">
-        <f>"Compte"</f>
+        <f t="shared" ref="B5:B13" si="0">"Compte"</f>
         <v>Compte</v>
       </c>
       <c r="C5" s="3" t="str">
@@ -805,7 +801,7 @@
         <v>AUTH-02</v>
       </c>
       <c r="B6" s="3" t="str">
-        <f>"Compte"</f>
+        <f t="shared" si="0"/>
         <v>Compte</v>
       </c>
       <c r="C6" s="3" t="str">
@@ -855,7 +851,7 @@
         <v>AUTH-03</v>
       </c>
       <c r="B7" s="3" t="str">
-        <f>"Compte"</f>
+        <f t="shared" si="0"/>
         <v>Compte</v>
       </c>
       <c r="C7" s="3" t="str">
@@ -905,7 +901,7 @@
         <v>AUTH-04</v>
       </c>
       <c r="B8" s="3" t="str">
-        <f>"Compte"</f>
+        <f t="shared" si="0"/>
         <v>Compte</v>
       </c>
       <c r="C8" s="3" t="str">
@@ -955,7 +951,7 @@
         <v>AUTH-05</v>
       </c>
       <c r="B9" s="3" t="str">
-        <f>"Compte"</f>
+        <f t="shared" si="0"/>
         <v>Compte</v>
       </c>
       <c r="C9" s="3" t="str">
@@ -1005,7 +1001,7 @@
         <v>AUTH-06</v>
       </c>
       <c r="B10" s="3" t="str">
-        <f>"Compte"</f>
+        <f t="shared" si="0"/>
         <v>Compte</v>
       </c>
       <c r="C10" s="3" t="str">
@@ -1055,7 +1051,7 @@
         <v>AUTH-07</v>
       </c>
       <c r="B11" s="3" t="str">
-        <f>"Compte"</f>
+        <f t="shared" si="0"/>
         <v>Compte</v>
       </c>
       <c r="C11" s="3" t="str">
@@ -1105,7 +1101,7 @@
         <v>AUTH-08</v>
       </c>
       <c r="B12" s="3" t="str">
-        <f>"Compte"</f>
+        <f t="shared" si="0"/>
         <v>Compte</v>
       </c>
       <c r="C12" s="3" t="str">
@@ -1155,7 +1151,7 @@
         <v>PROF-01</v>
       </c>
       <c r="B13" s="3" t="str">
-        <f>"Compte"</f>
+        <f t="shared" si="0"/>
         <v>Compte</v>
       </c>
       <c r="C13" s="3" t="str">
@@ -1205,7 +1201,7 @@
         <v>INF-01</v>
       </c>
       <c r="B14" s="4" t="str">
-        <f>"Informations"</f>
+        <f t="shared" ref="B14:B20" si="1">"Informations"</f>
         <v>Informations</v>
       </c>
       <c r="C14" s="4" t="str">
@@ -1255,7 +1251,7 @@
         <v>INF-02</v>
       </c>
       <c r="B15" s="4" t="str">
-        <f>"Informations"</f>
+        <f t="shared" si="1"/>
         <v>Informations</v>
       </c>
       <c r="C15" s="4" t="str">
@@ -1305,7 +1301,7 @@
         <v>INF-03</v>
       </c>
       <c r="B16" s="4" t="str">
-        <f>"Informations"</f>
+        <f t="shared" si="1"/>
         <v>Informations</v>
       </c>
       <c r="C16" s="4" t="str">
@@ -1355,7 +1351,7 @@
         <v>INF-04</v>
       </c>
       <c r="B17" s="4" t="str">
-        <f>"Informations"</f>
+        <f t="shared" si="1"/>
         <v>Informations</v>
       </c>
       <c r="C17" s="4" t="str">
@@ -1405,7 +1401,7 @@
         <v>INF-05</v>
       </c>
       <c r="B18" s="4" t="str">
-        <f>"Informations"</f>
+        <f t="shared" si="1"/>
         <v>Informations</v>
       </c>
       <c r="C18" s="4" t="str">
@@ -1455,7 +1451,7 @@
         <v>INF-06</v>
       </c>
       <c r="B19" s="4" t="str">
-        <f>"Informations"</f>
+        <f t="shared" si="1"/>
         <v>Informations</v>
       </c>
       <c r="C19" s="4" t="str">
@@ -1505,7 +1501,7 @@
         <v>INF-07</v>
       </c>
       <c r="B20" s="4" t="str">
-        <f>"Informations"</f>
+        <f t="shared" si="1"/>
         <v>Informations</v>
       </c>
       <c r="C20" s="4" t="str">
@@ -1555,7 +1551,7 @@
         <v>ACT-01</v>
       </c>
       <c r="B21" s="7" t="str">
-        <f>"Activités"</f>
+        <f t="shared" ref="B21:B28" si="2">"Activités"</f>
         <v>Activités</v>
       </c>
       <c r="C21" s="7" t="str">
@@ -1605,7 +1601,7 @@
         <v>ACT-02</v>
       </c>
       <c r="B22" s="7" t="str">
-        <f>"Activités"</f>
+        <f t="shared" si="2"/>
         <v>Activités</v>
       </c>
       <c r="C22" s="7" t="str">
@@ -1655,7 +1651,7 @@
         <v>ACT-03</v>
       </c>
       <c r="B23" s="7" t="str">
-        <f>"Activités"</f>
+        <f t="shared" si="2"/>
         <v>Activités</v>
       </c>
       <c r="C23" s="7" t="str">
@@ -1705,7 +1701,7 @@
         <v>ACT-04</v>
       </c>
       <c r="B24" s="7" t="str">
-        <f>"Activités"</f>
+        <f t="shared" si="2"/>
         <v>Activités</v>
       </c>
       <c r="C24" s="7" t="str">
@@ -1755,7 +1751,7 @@
         <v>ACT-05</v>
       </c>
       <c r="B25" s="7" t="str">
-        <f>"Activités"</f>
+        <f t="shared" si="2"/>
         <v>Activités</v>
       </c>
       <c r="C25" s="7" t="str">
@@ -1805,7 +1801,7 @@
         <v>ACT-06</v>
       </c>
       <c r="B26" s="7" t="str">
-        <f>"Activités"</f>
+        <f t="shared" si="2"/>
         <v>Activités</v>
       </c>
       <c r="C26" s="7" t="str">
@@ -1855,7 +1851,7 @@
         <v>ACT-07</v>
       </c>
       <c r="B27" s="7" t="str">
-        <f>"Activités"</f>
+        <f t="shared" si="2"/>
         <v>Activités</v>
       </c>
       <c r="C27" s="7" t="str">
@@ -1905,7 +1901,7 @@
         <v>ACT-08</v>
       </c>
       <c r="B28" s="7" t="str">
-        <f>"Activités"</f>
+        <f t="shared" si="2"/>
         <v>Activités</v>
       </c>
       <c r="C28" s="7" t="str">
@@ -1917,7 +1913,7 @@
         <v>Vérifier qu'un administrateur peut créer, modifier, désactiver puis supprimer une activité.</v>
       </c>
       <c r="E28" s="7" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" ref="E28:E38" si="3">"Utilisateur authentifié avec rôle Admin."</f>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F28" s="7" t="str">
@@ -1955,7 +1951,7 @@
         <v>ADM-01</v>
       </c>
       <c r="B29" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" ref="B29:B38" si="4">"Administration"</f>
         <v>Administration</v>
       </c>
       <c r="C29" s="5" t="str">
@@ -1967,7 +1963,7 @@
         <v>Vérifier qu'un administrateur peut créer une activité via le formulaire admin.</v>
       </c>
       <c r="E29" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F29" s="5" t="str">
@@ -2005,7 +2001,7 @@
         <v>ADM-02</v>
       </c>
       <c r="B30" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" si="4"/>
         <v>Administration</v>
       </c>
       <c r="C30" s="5" t="str">
@@ -2017,7 +2013,7 @@
         <v>Vérifier qu'un administrateur peut créer une information via le formulaire admin.</v>
       </c>
       <c r="E30" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F30" s="5" t="str">
@@ -2055,7 +2051,7 @@
         <v>ADM-03</v>
       </c>
       <c r="B31" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" si="4"/>
         <v>Administration</v>
       </c>
       <c r="C31" s="5" t="str">
@@ -2067,7 +2063,7 @@
         <v>Vérifier qu'un administrateur peut activer ou désactiver un contenu.</v>
       </c>
       <c r="E31" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F31" s="5" t="str">
@@ -2105,7 +2101,7 @@
         <v>ADM-04</v>
       </c>
       <c r="B32" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" si="4"/>
         <v>Administration</v>
       </c>
       <c r="C32" s="5" t="str">
@@ -2117,7 +2113,7 @@
         <v>Vérifier qu'un administrateur peut promouvoir, rétrograder ou désactiver un compte utilisateur.</v>
       </c>
       <c r="E32" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F32" s="5" t="str">
@@ -2155,7 +2151,7 @@
         <v>ADM-05</v>
       </c>
       <c r="B33" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" si="4"/>
         <v>Administration</v>
       </c>
       <c r="C33" s="5" t="str">
@@ -2167,7 +2163,7 @@
         <v>Vérifier que l'administration charge les jeux de données et respecte l'onglet demandé.</v>
       </c>
       <c r="E33" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F33" s="5" t="str">
@@ -2205,7 +2201,7 @@
         <v>ADM-06</v>
       </c>
       <c r="B34" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" si="4"/>
         <v>Administration</v>
       </c>
       <c r="C34" s="5" t="str">
@@ -2217,7 +2213,7 @@
         <v>Vérifier que le tri des activités dans l'administration change bien l'ordre affiché.</v>
       </c>
       <c r="E34" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F34" s="5" t="str">
@@ -2255,7 +2251,7 @@
         <v>ADM-07</v>
       </c>
       <c r="B35" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" si="4"/>
         <v>Administration</v>
       </c>
       <c r="C35" s="5" t="str">
@@ -2267,7 +2263,7 @@
         <v>Vérifier que les catégories sont réparties entre activités et informations.</v>
       </c>
       <c r="E35" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F35" s="5" t="str">
@@ -2305,7 +2301,7 @@
         <v>CAT-01</v>
       </c>
       <c r="B36" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" si="4"/>
         <v>Administration</v>
       </c>
       <c r="C36" s="5" t="str">
@@ -2317,7 +2313,7 @@
         <v>Vérifier qu'un administrateur peut consulter, créer et supprimer une catégorie.</v>
       </c>
       <c r="E36" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F36" s="5" t="str">
@@ -2355,7 +2351,7 @@
         <v>DIF-01</v>
       </c>
       <c r="B37" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" si="4"/>
         <v>Administration</v>
       </c>
       <c r="C37" s="5" t="str">
@@ -2367,7 +2363,7 @@
         <v>Vérifier que les niveaux de difficulté se chargent correctement dans le panneau admin.</v>
       </c>
       <c r="E37" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F37" s="5" t="str">
@@ -2405,7 +2401,7 @@
         <v>DIF-02</v>
       </c>
       <c r="B38" s="5" t="str">
-        <f>"Administration"</f>
+        <f t="shared" si="4"/>
         <v>Administration</v>
       </c>
       <c r="C38" s="5" t="str">
@@ -2417,7 +2413,7 @@
         <v>Vérifier qu'un administrateur peut créer, mettre à jour et supprimer un niveau de difficulté.</v>
       </c>
       <c r="E38" s="5" t="str">
-        <f>"Utilisateur authentifié avec rôle Admin."</f>
+        <f t="shared" si="3"/>
         <v>Utilisateur authentifié avec rôle Admin.</v>
       </c>
       <c r="F38" s="5" t="str">

</xml_diff>